<commit_message>
Updates for calibrated grid battery storage deployment
</commit_message>
<xml_diff>
--- a/InputData/elec/GBCGpUNR/Grid Bat Cap Growth per Unit Net Revenue.xlsx
+++ b/InputData/elec/GBCGpUNR/Grid Bat Cap Growth per Unit Net Revenue.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Desktop\EPS Models\SouthKorea EPS\InputData\elec\GBCGpUNR\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\South Korea\Models\eps-southkorea\InputData\elec\GBCGpUNR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDEA7FC1-CD97-4680-BE36-0481F1CD4C9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C81031D8-CA36-4495-BAAD-F1A0AA54070F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2604" yWindow="960" windowWidth="18660" windowHeight="12228" activeTab="1" xr2:uid="{7E47E401-4FF2-4F75-986A-BA871D3584BD}"/>
+    <workbookView xWindow="2700" yWindow="3060" windowWidth="43200" windowHeight="17145" activeTab="1" xr2:uid="{7E47E401-4FF2-4F75-986A-BA871D3584BD}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -435,7 +435,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1BF9ED0-8E48-4355-BDAD-C352BC3B92D2}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
@@ -467,9 +467,9 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="62.88671875" customWidth="1"/>
+    <col min="1" max="1" width="62.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="3" customFormat="1">
@@ -485,7 +485,7 @@
         <v>5</v>
       </c>
       <c r="B2">
-        <v>200</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -495,6 +495,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -638,22 +653,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{219152FF-ED81-4F5E-A116-61CA577ED93E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AA678E7-EBA2-4B97-BA43-1B14717CCBB3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14FE2E6F-14E7-405C-9661-491A200AA7D8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -669,21 +686,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AA678E7-EBA2-4B97-BA43-1B14717CCBB3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{219152FF-ED81-4F5E-A116-61CA577ED93E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update to unit for GBCGpUNR
</commit_message>
<xml_diff>
--- a/InputData/elec/GBCGpUNR/Grid Bat Cap Growth per Unit Net Revenue.xlsx
+++ b/InputData/elec/GBCGpUNR/Grid Bat Cap Growth per Unit Net Revenue.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\South Korea\Models\eps-southkorea\InputData\elec\GBCGpUNR\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-southkorea\InputData\elec\GBCGpUNR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C81031D8-CA36-4495-BAAD-F1A0AA54070F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7654E0D-0651-4226-A9AC-6A080B245C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2700" yWindow="3060" windowWidth="43200" windowHeight="17145" activeTab="1" xr2:uid="{7E47E401-4FF2-4F75-986A-BA871D3584BD}"/>
+    <workbookView xWindow="-24075" yWindow="1230" windowWidth="14400" windowHeight="8175" activeTab="1" xr2:uid="{7E47E401-4FF2-4F75-986A-BA871D3584BD}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -435,7 +435,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1BF9ED0-8E48-4355-BDAD-C352BC3B92D2}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
@@ -467,9 +467,9 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="62.85546875" customWidth="1"/>
+    <col min="1" max="1" width="62.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="3" customFormat="1">
@@ -485,7 +485,8 @@
         <v>5</v>
       </c>
       <c r="B2">
-        <v>50</v>
+        <f>1/7.5</f>
+        <v>0.13333333333333333</v>
       </c>
     </row>
   </sheetData>
@@ -495,18 +496,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -654,18 +655,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AA678E7-EBA2-4B97-BA43-1B14717CCBB3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{219152FF-ED81-4F5E-A116-61CA577ED93E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AA678E7-EBA2-4B97-BA43-1B14717CCBB3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>